<commit_message>
Corrige nome da coleção Alvimia para Alvimea
</commit_message>
<xml_diff>
--- a/produtos.xlsx
+++ b/produtos.xlsx
@@ -2275,7 +2275,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Alvimia</t>
+          <t>Alvimea</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2316,7 +2316,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Alvimia</t>
+          <t>Alvimea</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2357,7 +2357,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Alvimia</t>
+          <t>Alvimea</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza preços e cores dos produtos
Cores traduzidas para português e preços/custos revisados na planilha de produtos usada para gerar orçamentos.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/produtos.xlsx
+++ b/produtos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/raphaelsilvestre/EARE_Vendas/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/raphaelsilvestre/Documents/Claude/Projects/App Vendas - EARE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5111CBF8-39C8-9547-9E65-B5D133DE2982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7CBEC36-EB20-F648-95B1-397AF14C6EE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3360" yWindow="1800" windowWidth="29400" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,20 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$50</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -62,6 +49,9 @@
     <t>custo</t>
   </si>
   <si>
+    <t>quantidade</t>
+  </si>
+  <si>
     <t>Interna</t>
   </si>
   <si>
@@ -71,6 +61,9 @@
     <t>Mesa Centro</t>
   </si>
   <si>
+    <t>ambar</t>
+  </si>
+  <si>
     <t>Antares coffee table</t>
   </si>
   <si>
@@ -107,6 +100,9 @@
     <t>banco caramelo</t>
   </si>
   <si>
+    <t>marrom-preto</t>
+  </si>
+  <si>
     <t>banco café</t>
   </si>
   <si>
@@ -116,12 +112,18 @@
     <t>Poltrona</t>
   </si>
   <si>
+    <t>caramelo-vermelho</t>
+  </si>
+  <si>
     <t>Danica chair</t>
   </si>
   <si>
     <t>poltrona caramelo/vermelho</t>
   </si>
   <si>
+    <t>caramelo-cinza</t>
+  </si>
+  <si>
     <t>poltrona caramelo/cinza</t>
   </si>
   <si>
@@ -134,6 +136,9 @@
     <t>rosemary coffee table</t>
   </si>
   <si>
+    <t>trigo</t>
+  </si>
+  <si>
     <t>thyme side table</t>
   </si>
   <si>
@@ -338,7 +343,7 @@
     <t>Flexi Sun Lounger</t>
   </si>
   <si>
-    <t>Alvimia</t>
+    <t>Alvimea</t>
   </si>
   <si>
     <t>Sofá 3 lugares</t>
@@ -350,7 +355,10 @@
     <t>sofá 3 lugares</t>
   </si>
   <si>
-    <t>Sofá 1 lugar</t>
+    <t>Poltrona Alvimea</t>
+  </si>
+  <si>
+    <t>Bambu Natural c/ estofado off white</t>
   </si>
   <si>
     <t>Koloni Sofa</t>
@@ -377,44 +385,27 @@
     <t>mesa</t>
   </si>
   <si>
-    <t>quantidade</t>
-  </si>
-  <si>
-    <t>ambar</t>
-  </si>
-  <si>
-    <t>marrom escuro</t>
-  </si>
-  <si>
-    <t>caramelo</t>
-  </si>
-  <si>
-    <t>caramelo-vermelho</t>
-  </si>
-  <si>
-    <t>caramelo-cinza</t>
-  </si>
-  <si>
-    <t>trigo</t>
-  </si>
-  <si>
-    <t>N/D</t>
-  </si>
-  <si>
-    <t>marrom-preto</t>
+    <t>Bambu Natural</t>
+  </si>
+  <si>
+    <t>capim dourado</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
-  </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -442,10 +433,8 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -754,11 +743,12 @@
     <col min="1" max="1" width="6.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.83203125" customWidth="1"/>
+    <col min="4" max="4" width="28.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20.5" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="23.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
@@ -787,1427 +777,1427 @@
         <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>113</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>114</v>
+        <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2">
+        <v>14</v>
+      </c>
+      <c r="G2" s="2">
         <v>3870</v>
       </c>
       <c r="H2" s="2">
         <v>1074.57</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D3" t="s">
-        <v>114</v>
+        <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3">
+        <v>17</v>
+      </c>
+      <c r="G3" s="2">
         <v>3110</v>
       </c>
       <c r="H3" s="2">
         <v>752.93</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D4" t="s">
-        <v>114</v>
+        <v>12</v>
       </c>
       <c r="E4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G4">
+        <v>20</v>
+      </c>
+      <c r="G4" s="2">
         <v>1990</v>
       </c>
       <c r="H4" s="2">
         <v>451.77</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4">
         <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="E5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F5" t="s">
-        <v>22</v>
-      </c>
-      <c r="G5">
+        <v>24</v>
+      </c>
+      <c r="G5" s="2">
         <v>2970</v>
       </c>
       <c r="H5" s="2">
         <v>557.86</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D6" t="s">
-        <v>121</v>
+        <v>25</v>
       </c>
       <c r="E6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F6" t="s">
-        <v>23</v>
-      </c>
-      <c r="G6">
+        <v>26</v>
+      </c>
+      <c r="G6" s="2">
         <v>2970</v>
       </c>
       <c r="H6" s="2">
         <v>557.86</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6">
         <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D7" t="s">
-        <v>117</v>
+        <v>29</v>
       </c>
       <c r="E7" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F7" t="s">
-        <v>27</v>
-      </c>
-      <c r="G7">
+        <v>31</v>
+      </c>
+      <c r="G7" s="2">
         <v>3540</v>
       </c>
       <c r="H7" s="2">
         <v>729.55</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7">
         <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C8" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D8" t="s">
-        <v>118</v>
+        <v>32</v>
       </c>
       <c r="E8" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F8" t="s">
-        <v>28</v>
-      </c>
-      <c r="G8">
+        <v>33</v>
+      </c>
+      <c r="G8" s="2">
         <v>3540</v>
       </c>
       <c r="H8" s="2">
         <v>537.05999999999995</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8">
         <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="C9" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D9" t="s">
-        <v>114</v>
+        <v>12</v>
       </c>
       <c r="E9" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="F9" t="s">
-        <v>12</v>
-      </c>
-      <c r="G9">
+        <v>14</v>
+      </c>
+      <c r="G9" s="2">
         <v>4180</v>
       </c>
       <c r="H9" s="2">
         <v>816.09</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9">
         <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="C10" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D10" t="s">
-        <v>119</v>
+        <v>37</v>
       </c>
       <c r="E10" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="F10" t="s">
-        <v>12</v>
-      </c>
-      <c r="G10">
+        <v>14</v>
+      </c>
+      <c r="G10" s="2">
         <v>4180</v>
       </c>
       <c r="H10" s="2">
         <v>651.46</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10">
         <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="C11" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D11" t="s">
-        <v>114</v>
+        <v>12</v>
       </c>
       <c r="E11" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="F11" t="s">
-        <v>18</v>
-      </c>
-      <c r="G11">
+        <v>20</v>
+      </c>
+      <c r="G11" s="2">
         <v>1490</v>
       </c>
       <c r="H11" s="2">
         <v>486.43</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11">
         <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B12" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="C12" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D12" t="s">
-        <v>119</v>
+        <v>37</v>
       </c>
       <c r="E12" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="F12" t="s">
-        <v>18</v>
-      </c>
-      <c r="G12">
+        <v>20</v>
+      </c>
+      <c r="G12" s="2">
         <v>1490</v>
       </c>
       <c r="H12" s="2">
         <v>458.87</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12">
         <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B13" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C13" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D13" t="s">
-        <v>114</v>
+        <v>12</v>
       </c>
       <c r="E13" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="F13" t="s">
-        <v>35</v>
-      </c>
-      <c r="G13">
+        <v>41</v>
+      </c>
+      <c r="G13" s="2">
         <v>1780</v>
       </c>
       <c r="H13" s="2">
         <v>569.36</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13">
         <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B14" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C14" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D14" t="s">
-        <v>119</v>
+        <v>37</v>
       </c>
       <c r="E14" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="F14" t="s">
-        <v>35</v>
-      </c>
-      <c r="G14">
+        <v>41</v>
+      </c>
+      <c r="G14" s="2">
         <v>1780</v>
       </c>
       <c r="H14" s="2">
         <v>569.36</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14">
         <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B15" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C15" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="D15" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="E15" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="F15" t="s">
-        <v>38</v>
-      </c>
-      <c r="G15">
+        <v>44</v>
+      </c>
+      <c r="G15" s="2">
         <v>3650</v>
       </c>
       <c r="H15" s="2">
         <v>996.91</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15">
         <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B16" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C16" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="D16" t="s">
-        <v>114</v>
+        <v>12</v>
       </c>
       <c r="E16" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="F16" t="s">
-        <v>38</v>
-      </c>
-      <c r="G16">
+        <v>44</v>
+      </c>
+      <c r="G16" s="2">
         <v>3650</v>
       </c>
       <c r="H16" s="2">
         <v>996.91</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16">
         <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B17" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C17" t="s">
-        <v>39</v>
-      </c>
-      <c r="D17" t="s">
-        <v>116</v>
+        <v>45</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>121</v>
       </c>
       <c r="E17" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="F17" t="s">
-        <v>41</v>
-      </c>
-      <c r="G17">
+        <v>47</v>
+      </c>
+      <c r="G17" s="2">
         <v>13460</v>
       </c>
       <c r="H17" s="2">
         <v>4097.01</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17">
         <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B18" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C18" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="D18" t="s">
-        <v>114</v>
+        <v>12</v>
       </c>
       <c r="E18" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="F18" t="s">
-        <v>41</v>
-      </c>
-      <c r="G18">
+        <v>47</v>
+      </c>
+      <c r="G18" s="2">
         <v>13890</v>
       </c>
       <c r="H18" s="2">
         <v>4097.01</v>
       </c>
-      <c r="I18" s="1">
+      <c r="I18">
         <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B19" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C19" t="s">
-        <v>42</v>
-      </c>
-      <c r="D19" t="s">
-        <v>116</v>
+        <v>48</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>121</v>
       </c>
       <c r="E19" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="F19" t="s">
-        <v>44</v>
-      </c>
-      <c r="G19">
+        <v>50</v>
+      </c>
+      <c r="G19" s="2">
         <v>3590</v>
       </c>
       <c r="H19" s="2">
         <v>1026.6099999999999</v>
       </c>
-      <c r="I19" s="1">
+      <c r="I19">
         <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B20" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C20" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="D20" t="s">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="E20" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="F20" t="s">
-        <v>44</v>
-      </c>
-      <c r="G20">
+        <v>50</v>
+      </c>
+      <c r="G20" s="2">
         <v>3790</v>
       </c>
       <c r="H20" s="2">
         <v>4195.33</v>
       </c>
-      <c r="I20" s="1">
+      <c r="I20">
         <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B21" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="C21" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="D21" t="s">
-        <v>119</v>
+        <v>37</v>
       </c>
       <c r="E21" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="F21" t="s">
-        <v>38</v>
-      </c>
-      <c r="G21">
+        <v>44</v>
+      </c>
+      <c r="G21" s="2">
         <v>3290</v>
       </c>
       <c r="H21" s="2">
         <v>1026.6099999999999</v>
       </c>
-      <c r="I21" s="1">
+      <c r="I21">
         <v>4</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B22" t="s">
+        <v>51</v>
+      </c>
+      <c r="C22" t="s">
         <v>45</v>
       </c>
-      <c r="C22" t="s">
-        <v>39</v>
-      </c>
       <c r="D22" t="s">
-        <v>119</v>
+        <v>37</v>
       </c>
       <c r="E22" t="s">
+        <v>53</v>
+      </c>
+      <c r="F22" t="s">
         <v>47</v>
       </c>
-      <c r="F22" t="s">
-        <v>41</v>
-      </c>
-      <c r="G22">
+      <c r="G22" s="2">
         <v>12220</v>
       </c>
       <c r="H22" s="2">
         <v>4195.32</v>
       </c>
-      <c r="I22" s="1">
+      <c r="I22">
         <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B23" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="C23" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="D23" t="s">
-        <v>114</v>
+        <v>12</v>
       </c>
       <c r="E23" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="F23" t="s">
-        <v>38</v>
-      </c>
-      <c r="G23">
+        <v>44</v>
+      </c>
+      <c r="G23" s="2">
         <v>3305</v>
       </c>
       <c r="H23" s="2">
         <v>1015.11</v>
       </c>
-      <c r="I23" s="1">
+      <c r="I23">
         <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B24" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="C24" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="D24" t="s">
-        <v>114</v>
+        <v>12</v>
       </c>
       <c r="E24" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="F24" t="s">
-        <v>41</v>
-      </c>
-      <c r="G24">
+        <v>47</v>
+      </c>
+      <c r="G24" s="2">
         <v>12220</v>
       </c>
       <c r="H24" s="2">
         <v>3128.03</v>
       </c>
-      <c r="I24" s="1">
+      <c r="I24">
         <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B25" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="C25" t="s">
-        <v>36</v>
-      </c>
-      <c r="D25" t="s">
-        <v>116</v>
+        <v>42</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>121</v>
       </c>
       <c r="E25" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="F25" t="s">
-        <v>38</v>
-      </c>
-      <c r="G25">
+        <v>44</v>
+      </c>
+      <c r="G25" s="2">
         <v>3170</v>
       </c>
       <c r="H25" s="2">
         <v>4290.71</v>
       </c>
-      <c r="I25" s="1">
+      <c r="I25">
         <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B26" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="C26" t="s">
-        <v>39</v>
-      </c>
-      <c r="D26" t="s">
-        <v>116</v>
+        <v>45</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>121</v>
       </c>
       <c r="E26" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="F26" t="s">
-        <v>54</v>
-      </c>
-      <c r="G26">
+        <v>60</v>
+      </c>
+      <c r="G26" s="2">
         <v>9110</v>
       </c>
       <c r="H26" s="2">
         <v>1381.67</v>
       </c>
-      <c r="I26" s="1">
+      <c r="I26">
         <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B27" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C27" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="D27" t="s">
-        <v>114</v>
+        <v>12</v>
       </c>
       <c r="E27" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="F27" t="s">
-        <v>58</v>
-      </c>
-      <c r="G27">
+        <v>64</v>
+      </c>
+      <c r="G27" s="2">
         <v>14890</v>
       </c>
       <c r="H27" s="2">
         <v>674.62</v>
       </c>
-      <c r="I27" s="1">
+      <c r="I27">
         <v>32</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B28" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C28" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="D28" t="s">
-        <v>114</v>
+        <v>12</v>
       </c>
       <c r="E28" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="F28" t="s">
-        <v>60</v>
-      </c>
-      <c r="G28">
+        <v>66</v>
+      </c>
+      <c r="G28" s="2">
         <v>9980</v>
       </c>
       <c r="H28" s="2">
         <v>2403.81</v>
       </c>
-      <c r="I28" s="1">
+      <c r="I28">
         <v>3</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B29" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C29" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="D29" t="s">
-        <v>114</v>
+        <v>12</v>
       </c>
       <c r="E29" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="F29" t="s">
-        <v>63</v>
-      </c>
-      <c r="G29">
+        <v>69</v>
+      </c>
+      <c r="G29" s="2">
         <v>1980</v>
       </c>
       <c r="H29" s="2">
         <v>880.54</v>
       </c>
-      <c r="I29" s="1">
+      <c r="I29">
         <v>22</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B30" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C30" t="s">
-        <v>64</v>
-      </c>
-      <c r="D30" t="s">
-        <v>116</v>
+        <v>70</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>121</v>
       </c>
       <c r="E30" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="F30" t="s">
-        <v>66</v>
-      </c>
-      <c r="G30">
+        <v>72</v>
+      </c>
+      <c r="G30" s="2">
         <v>1780</v>
       </c>
       <c r="H30" s="2">
         <v>1422.02</v>
       </c>
-      <c r="I30" s="1">
+      <c r="I30">
         <v>3</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B31" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C31" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="D31" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E31" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="F31" t="s">
-        <v>69</v>
-      </c>
-      <c r="G31">
+        <v>75</v>
+      </c>
+      <c r="G31" s="2">
         <v>15990</v>
       </c>
       <c r="H31" s="2">
         <v>759.06</v>
       </c>
-      <c r="I31" s="1">
+      <c r="I31">
         <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B32" t="s">
+        <v>73</v>
+      </c>
+      <c r="C32" t="s">
         <v>67</v>
       </c>
-      <c r="C32" t="s">
-        <v>61</v>
-      </c>
       <c r="D32" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E32" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="F32" t="s">
-        <v>71</v>
-      </c>
-      <c r="G32">
+        <v>77</v>
+      </c>
+      <c r="G32" s="2">
         <v>2680</v>
       </c>
       <c r="H32" s="2">
         <v>3921.51</v>
       </c>
-      <c r="I32" s="1">
+      <c r="I32">
         <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B33" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C33" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D33" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E33" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="F33" t="s">
-        <v>73</v>
-      </c>
-      <c r="G33">
+        <v>79</v>
+      </c>
+      <c r="G33" s="2">
         <v>12260</v>
       </c>
       <c r="H33" s="2">
         <v>643.17999999999995</v>
       </c>
-      <c r="I33" s="1">
+      <c r="I33">
         <v>12</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B34" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="C34" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="D34" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E34" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="F34" t="s">
-        <v>77</v>
-      </c>
-      <c r="G34">
+        <v>83</v>
+      </c>
+      <c r="G34" s="2">
         <v>4990</v>
       </c>
       <c r="H34" s="2">
         <v>683.09</v>
       </c>
-      <c r="I34" s="1">
+      <c r="I34">
         <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B35" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="C35" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="D35" t="s">
-        <v>114</v>
+        <v>12</v>
       </c>
       <c r="E35" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="F35" t="s">
-        <v>77</v>
-      </c>
-      <c r="G35">
+        <v>83</v>
+      </c>
+      <c r="G35" s="2">
         <v>5110</v>
       </c>
       <c r="H35" s="2">
         <v>683.09</v>
       </c>
-      <c r="I35" s="1">
+      <c r="I35">
         <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B36" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="C36" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="D36" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E36" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="F36" t="s">
-        <v>80</v>
-      </c>
-      <c r="G36">
+        <v>86</v>
+      </c>
+      <c r="G36" s="2">
         <v>2110</v>
       </c>
       <c r="H36" s="2">
         <v>814.67</v>
       </c>
-      <c r="I36" s="1">
+      <c r="I36">
         <v>12</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B37" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="C37" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="D37" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="E37" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="F37" t="s">
-        <v>82</v>
-      </c>
-      <c r="G37">
+        <v>88</v>
+      </c>
+      <c r="G37" s="2">
         <v>2110</v>
       </c>
       <c r="H37" s="2">
         <v>814.67</v>
       </c>
-      <c r="I37" s="1">
+      <c r="I37">
         <v>12</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="B38" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C38" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="D38" t="s">
         <v>120</v>
       </c>
       <c r="E38" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="F38" t="s">
-        <v>85</v>
-      </c>
-      <c r="G38">
+        <v>91</v>
+      </c>
+      <c r="G38" s="2">
         <v>8110</v>
       </c>
       <c r="H38" s="2">
         <v>1130.1300000000001</v>
       </c>
-      <c r="I38" s="1">
+      <c r="I38">
         <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="B39" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C39" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="D39" t="s">
         <v>120</v>
       </c>
       <c r="E39" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="F39" t="s">
-        <v>87</v>
-      </c>
-      <c r="G39">
+        <v>93</v>
+      </c>
+      <c r="G39" s="2">
         <v>1940</v>
       </c>
       <c r="H39" s="2">
         <v>665.75</v>
       </c>
-      <c r="I39" s="1">
+      <c r="I39">
         <v>12</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="B40" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C40" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="D40" t="s">
         <v>120</v>
       </c>
       <c r="E40" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="F40" t="s">
-        <v>90</v>
-      </c>
-      <c r="G40">
-        <v>5990</v>
+        <v>96</v>
+      </c>
+      <c r="G40" s="2">
+        <v>7150</v>
       </c>
       <c r="H40" s="2">
         <v>1036.01</v>
       </c>
-      <c r="I40" s="1">
+      <c r="I40">
         <v>6</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="B41" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C41" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="D41" t="s">
         <v>120</v>
       </c>
       <c r="E41" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="F41" t="s">
-        <v>93</v>
-      </c>
-      <c r="G41">
-        <v>6530</v>
+        <v>99</v>
+      </c>
+      <c r="G41" s="2">
+        <v>7600</v>
       </c>
       <c r="H41" s="2">
         <v>1228.78</v>
       </c>
-      <c r="I41" s="1">
+      <c r="I41">
         <v>3</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="B42" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="C42" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="D42" t="s">
         <v>120</v>
       </c>
       <c r="E42" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F42" t="s">
-        <v>85</v>
-      </c>
-      <c r="G42">
-        <v>8230</v>
+        <v>91</v>
+      </c>
+      <c r="G42" s="2">
+        <v>9450</v>
       </c>
       <c r="H42" s="2">
         <v>937.32</v>
       </c>
-      <c r="I42" s="1">
+      <c r="I42">
         <v>18</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="B43" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="C43" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="D43" t="s">
         <v>120</v>
       </c>
       <c r="E43" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="F43" t="s">
-        <v>87</v>
-      </c>
-      <c r="G43">
+        <v>93</v>
+      </c>
+      <c r="G43" s="2">
         <v>2600</v>
       </c>
       <c r="H43" s="2">
         <v>1448.63</v>
       </c>
-      <c r="I43" s="1">
+      <c r="I43">
         <v>2</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="B44" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="C44" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D44" t="s">
         <v>120</v>
       </c>
       <c r="E44" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="F44" t="s">
-        <v>98</v>
-      </c>
-      <c r="G44">
-        <v>5230</v>
+        <v>104</v>
+      </c>
+      <c r="G44" s="2">
+        <v>5550</v>
       </c>
       <c r="H44" s="2">
         <v>1062.8</v>
       </c>
-      <c r="I44" s="1">
+      <c r="I44">
         <v>4</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="B45" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="C45" t="s">
-        <v>88</v>
-      </c>
-      <c r="D45" t="s">
+        <v>94</v>
+      </c>
+      <c r="D45" s="1" t="s">
         <v>120</v>
       </c>
       <c r="E45" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="F45" t="s">
-        <v>90</v>
-      </c>
-      <c r="G45">
-        <v>11525</v>
+        <v>96</v>
+      </c>
+      <c r="G45" s="2">
+        <v>13850</v>
       </c>
       <c r="H45" s="2">
         <v>2145.7399999999998</v>
       </c>
-      <c r="I45" s="1">
+      <c r="I45">
         <v>3</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="B46" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="C46" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="D46" t="s">
-        <v>120</v>
+        <v>111</v>
       </c>
       <c r="E46" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="F46" t="s">
-        <v>103</v>
-      </c>
-      <c r="G46">
-        <v>13000</v>
+        <v>109</v>
+      </c>
+      <c r="G46" s="2">
+        <v>15200</v>
       </c>
       <c r="H46" s="2">
         <v>2880.69</v>
       </c>
-      <c r="I46" s="1">
+      <c r="I46">
         <v>3</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="B47" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="C47" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="D47" t="s">
-        <v>120</v>
+        <v>111</v>
       </c>
       <c r="E47" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="F47" t="s">
-        <v>106</v>
-      </c>
-      <c r="G47">
-        <v>5250</v>
+        <v>113</v>
+      </c>
+      <c r="G47" s="2">
+        <v>6200</v>
       </c>
       <c r="H47" s="2">
         <v>368.75</v>
       </c>
-      <c r="I47" s="1">
+      <c r="I47">
         <v>6</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="B48" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="C48" t="s">
-        <v>30</v>
-      </c>
-      <c r="D48" t="s">
+        <v>35</v>
+      </c>
+      <c r="D48" s="1" t="s">
         <v>120</v>
       </c>
       <c r="E48" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="F48" t="s">
-        <v>12</v>
-      </c>
-      <c r="G48">
-        <v>5270</v>
+        <v>14</v>
+      </c>
+      <c r="G48" s="2">
+        <v>6150</v>
       </c>
       <c r="H48" s="2">
         <v>1119.77</v>
       </c>
-      <c r="I48" s="1">
+      <c r="I48">
         <v>3</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="B49" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="C49" t="s">
-        <v>61</v>
-      </c>
-      <c r="D49" t="s">
+        <v>67</v>
+      </c>
+      <c r="D49" s="1" t="s">
         <v>120</v>
       </c>
       <c r="E49" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="F49" t="s">
-        <v>110</v>
-      </c>
-      <c r="G49">
+        <v>117</v>
+      </c>
+      <c r="G49" s="2">
         <v>2650</v>
       </c>
       <c r="H49" s="2">
         <v>870.31</v>
       </c>
-      <c r="I49" s="1">
+      <c r="I49">
         <v>8</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="B50" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="C50" t="s">
-        <v>75</v>
-      </c>
-      <c r="D50" t="s">
+        <v>81</v>
+      </c>
+      <c r="D50" s="1" t="s">
         <v>120</v>
       </c>
       <c r="E50" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="F50" t="s">
-        <v>112</v>
-      </c>
-      <c r="G50">
+        <v>119</v>
+      </c>
+      <c r="G50" s="2">
         <v>3120</v>
       </c>
       <c r="H50" s="2">
         <v>878.35</v>
       </c>
-      <c r="I50" s="1">
+      <c r="I50">
         <v>2</v>
       </c>
     </row>

</xml_diff>